<commit_message>
chore: weekly briefing 2026-09-14 14:03Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-14.xlsx
+++ b/public/reports/weekly_briefing/2026-09-14.xlsx
@@ -932,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12.9" customWidth="1" style="15" min="1" max="1"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14 22:50 KST</t>
+          <t>2026-09-14 23:03 KST</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>AI 속도조절론 부각에 따른 반도체 급락과 외국인 대규모 매도</t>
+          <t>미국발 AI 속도조절론과 외국인 대규모 매도세에 따른 코스피 급락</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="G33" s="17" t="inlineStr">
         <is>
-          <t>미국 증시는 CPI 예상치 부합으로 상승했으나, 국내 증시는 'AI 속도조절론'이 부각되며 반도체 중심의 외국인 매도세가 쏟아져 급락함.</t>
+          <t>미국 증시의 기술주 반등과 CPI 예상치 부합에도 불구하고, 국내 증시는 미국발 'AI 속도조절론'이 부각되며 반도체 대형주 중심의 외국인 매도세가 쏟아져 급락함.</t>
         </is>
       </c>
     </row>
@@ -1720,21 +1720,21 @@
     <row r="37" ht="31" customHeight="1" s="15">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>- 미국 8월 CPI는 3.4%로 예상치에 부합했으나, 미시간대 소비자심리지수는 47.8로 예상치(51.0)를 하회하며 매크로 환경의 불확실성이 잔존함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="15">
+          <t>- 미국 8월 소비자물가지수(CPI)는 전년 대비 3.4%로 예상치에 부합하며 인플레이션 둔화 경로를 재확인했으나, 미시간대 소비자심리지수는 47.8로 예상치(51.0)를 하회하며 소비 심리 위축을 시사함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="31" customHeight="1" s="15">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>- 수급 측면에서 외국인은 전기·전자 섹터에 매도를 집중하며 코스피 3.3조 원 순매도를 기록, 지수 하락의 핵심 동인으로 작용함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="15">
+          <t>- 수급 측면에서 코스피는 외국인 -32,875억 원, 기관 -11,742억 원의 동반 매도세가 지수를 끌어내렸으며, 특히 전기·전자 섹터에 외국인 매물이 집중됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="31" customHeight="1" s="15">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>- 매크로 지표보다 AI 산업에 대한 센티먼트 변화가 시장 수급을 지배하는 국면임.</t>
+          <t>- 매크로 환경의 불확실성과 반도체 섹터에 대한 수급 이탈이 겹치며 지수 하락을 주도했으므로, 향후 외국인 매도세 진정 여부와 수출입 확정치가 증시 반등의 핵심 변수가 될 것임.</t>
         </is>
       </c>
     </row>
@@ -3082,197 +3082,141 @@
     <row r="93" ht="15" customHeight="1" s="15">
       <c r="A93" s="17" t="inlineStr">
         <is>
-          <t>- 코스피는 외국인의 3.3조 원 규모 매도세가 쏟아지며 전일 대비 3.26% 급락한 6684.37에 마감함.</t>
+          <t>- 코스피는 외국인의 3.3조 원 규모 대규모 매도세가 쏟아지며 전일 대비 3.26% 급락한 6684.37에 마감함.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="15">
       <c r="A94" s="17" t="inlineStr">
         <is>
-          <t>- 코스닥 역시 투자 심리 위축으로 1.69% 하락하며 동반 약세를 보임.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="15" customHeight="1" s="15">
+          <t>- 코스닥 역시 1.69% 하락하며 투자 심리가 크게 위축됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="31" customHeight="1" s="15">
       <c r="A95" s="17" t="inlineStr">
         <is>
-          <t>- 미국발 'AI 속도조절론'이 부각되면서 전기·전자 섹터에 외국인 매물이 집중되어 지수 하락을 주도함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="15" customHeight="1" s="15">
+          <t>- 전기·전자 섹터는 미국발 'AI 속도조절론'이 부각되면서 삼성전자와 SK하이닉스에 외국인 매물이 집중되어 각각 3%와 6%대 급락하며 지수 하락의 핵심 원인이 됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="31" customHeight="1" s="15">
       <c r="A96" s="17" t="inlineStr">
         <is>
-          <t>- 반면 방산 및 조선 섹터는 연이은 수주 계약 성공으로 상대적 견조함을 유지함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97"/>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
+          <t>- 시장 전반의 약세 속에서도 운송·창고 섹터는 중동 지정학적 리스크에 따른 해운 운임 상승 기대감과 통합 항공사 출범 이슈로 견조한 흐름을 보임.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1" s="15">
+      <c r="A97" s="17" t="inlineStr">
+        <is>
+          <t>- 외국인과 기관의 동반 매도세가 지수 하락을 주도함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98"/>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>섹터·테마 흐름</t>
         </is>
       </c>
-      <c r="C98" s="3" t="inlineStr"/>
-      <c r="D98" s="3" t="inlineStr"/>
-      <c r="E98" s="3" t="inlineStr"/>
-      <c r="F98" s="3" t="inlineStr"/>
-      <c r="G98" s="3" t="inlineStr"/>
-      <c r="H98" s="3" t="inlineStr"/>
-      <c r="I98" s="3" t="inlineStr"/>
-      <c r="J98" s="3" t="inlineStr"/>
-      <c r="K98" s="3" t="inlineStr"/>
-    </row>
-    <row r="99" ht="15" customHeight="1" s="15">
-      <c r="A99" s="17" t="inlineStr">
-        <is>
-          <t>- 전기·전자 섹터는 AI 관련 우려로 외국인 매물이 집중되며 급락세 지속.</t>
-        </is>
-      </c>
+      <c r="C99" s="3" t="inlineStr"/>
+      <c r="D99" s="3" t="inlineStr"/>
+      <c r="E99" s="3" t="inlineStr"/>
+      <c r="F99" s="3" t="inlineStr"/>
+      <c r="G99" s="3" t="inlineStr"/>
+      <c r="H99" s="3" t="inlineStr"/>
+      <c r="I99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="inlineStr"/>
+      <c r="K99" s="3" t="inlineStr"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="15">
       <c r="A100" s="17" t="inlineStr">
         <is>
-          <t>- 운송·창고 및 오락·문화 섹터는 개별 이슈와 수급 유입으로 방어적 흐름을 보임.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101"/>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
+          <t>- 전기·전자 섹터는 미국발 AI 속도조절론 부각으로 외국인 매물이 집중되며 급락함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="15">
+      <c r="A101" s="17" t="inlineStr">
+        <is>
+          <t>- 운송·창고 섹터는 지정학적 리스크와 통합 항공사 이슈로 견조한 흐름을 보임.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1" s="15">
+      <c r="A102" s="17" t="inlineStr">
+        <is>
+          <t>- 오락·문화 섹터는 글로벌 IP 파워 기대감으로 상승하며 방어적 성격을 보임.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103"/>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>주간 촉매 타임라인</t>
         </is>
       </c>
-      <c r="C102" s="3" t="inlineStr"/>
-      <c r="D102" s="3" t="inlineStr"/>
-      <c r="E102" s="3" t="inlineStr"/>
-      <c r="F102" s="3" t="inlineStr"/>
-      <c r="G102" s="3" t="inlineStr"/>
-      <c r="H102" s="3" t="inlineStr"/>
-      <c r="I102" s="3" t="inlineStr"/>
-      <c r="J102" s="18" t="inlineStr">
+      <c r="C104" s="3" t="inlineStr"/>
+      <c r="D104" s="3" t="inlineStr"/>
+      <c r="E104" s="3" t="inlineStr"/>
+      <c r="F104" s="3" t="inlineStr"/>
+      <c r="G104" s="3" t="inlineStr"/>
+      <c r="H104" s="3" t="inlineStr"/>
+      <c r="I104" s="3" t="inlineStr"/>
+      <c r="J104" s="18" t="inlineStr">
         <is>
           <t>등락률 = 주간 누적</t>
         </is>
       </c>
-      <c r="K102" s="3" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="4" t="inlineStr">
+      <c r="K104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>날짜</t>
         </is>
       </c>
-      <c r="B103" s="4" t="inlineStr">
+      <c r="B105" s="4" t="inlineStr">
         <is>
           <t>종목명</t>
         </is>
       </c>
-      <c r="C103" s="4" t="inlineStr">
+      <c r="C105" s="4" t="inlineStr">
         <is>
           <t>시장</t>
         </is>
       </c>
-      <c r="D103" s="4" t="inlineStr">
+      <c r="D105" s="4" t="inlineStr">
         <is>
           <t>섹터명</t>
         </is>
       </c>
-      <c r="E103" s="4" t="inlineStr">
+      <c r="E105" s="4" t="inlineStr">
         <is>
           <t>별점</t>
         </is>
       </c>
-      <c r="F103" s="4" t="inlineStr">
+      <c r="F105" s="4" t="inlineStr">
         <is>
           <t>등락률(%)</t>
         </is>
       </c>
-      <c r="G103" s="4" t="inlineStr">
+      <c r="G105" s="4" t="inlineStr">
         <is>
           <t>핵심 촉매</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="31" customHeight="1" s="15">
-      <c r="A104" s="31" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B104" s="17" t="inlineStr">
-        <is>
-          <t>인피니트헬스케어</t>
-        </is>
-      </c>
-      <c r="C104" s="31" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D104" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E104" s="14" t="inlineStr">
-        <is>
-          <t>★★★★★</t>
-        </is>
-      </c>
-      <c r="F104" s="28" t="n">
-        <v>30</v>
-      </c>
-      <c r="G104" s="17" t="inlineStr">
-        <is>
-          <t>654억 원 규모의 대규모 현금배당 계획 발표.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="15" customHeight="1" s="15">
-      <c r="A105" s="31" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B105" s="31" t="inlineStr">
-        <is>
-          <t>한국첨단소재</t>
-        </is>
-      </c>
-      <c r="C105" s="31" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D105" s="35" t="inlineStr">
-        <is>
-          <t>전기·전자</t>
-        </is>
-      </c>
-      <c r="E105" s="14" t="inlineStr">
-        <is>
-          <t>★★★★★</t>
-        </is>
-      </c>
-      <c r="F105" s="28" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="G105" s="17" t="inlineStr">
-        <is>
-          <t>차세대 광통신 기술 검증 및 양자통신 클러스터 참여.</t>
         </is>
       </c>
     </row>
@@ -3284,17 +3228,17 @@
       </c>
       <c r="B106" s="17" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>인피니트헬스케어</t>
         </is>
       </c>
       <c r="C106" s="31" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D106" s="35" t="inlineStr">
         <is>
-          <t>운송장비·부품</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E106" s="14" t="inlineStr">
@@ -3303,11 +3247,11 @@
         </is>
       </c>
       <c r="F106" s="28" t="n">
-        <v>5.4</v>
+        <v>30</v>
       </c>
       <c r="G106" s="17" t="inlineStr">
         <is>
-          <t>K9 자주포 및 천무 등 연이은 수출 계약 성공.</t>
+          <t>654억 원 규모의 대규모 현금배당 계획 발표.</t>
         </is>
       </c>
     </row>
@@ -3319,134 +3263,197 @@
       </c>
       <c r="B107" s="31" t="inlineStr">
         <is>
+          <t>한국첨단소재</t>
+        </is>
+      </c>
+      <c r="C107" s="31" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D107" s="35" t="inlineStr">
+        <is>
+          <t>전기·전자</t>
+        </is>
+      </c>
+      <c r="E107" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="F107" s="28" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="G107" s="17" t="inlineStr">
+        <is>
+          <t>차세대 광통신 기술 검증 및 양자통신 클러스터 참여.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="31" customHeight="1" s="15">
+      <c r="A108" s="31" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B108" s="17" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C108" s="31" t="inlineStr">
+        <is>
+          <t>KOSPI</t>
+        </is>
+      </c>
+      <c r="D108" s="35" t="inlineStr">
+        <is>
+          <t>운송장비·부품</t>
+        </is>
+      </c>
+      <c r="E108" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="F108" s="28" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G108" s="17" t="inlineStr">
+        <is>
+          <t>K9 자주포 및 천무 등 연이은 수출 계약 성공.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="15">
+      <c r="A109" s="31" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B109" s="31" t="inlineStr">
+        <is>
           <t>삼성중공업</t>
         </is>
       </c>
-      <c r="C107" s="31" t="inlineStr">
+      <c r="C109" s="31" t="inlineStr">
         <is>
           <t>KOSPI</t>
         </is>
       </c>
-      <c r="D107" s="35" t="inlineStr">
+      <c r="D109" s="35" t="inlineStr">
         <is>
           <t>운송장비·부품</t>
         </is>
       </c>
-      <c r="E107" s="14" t="inlineStr">
+      <c r="E109" s="14" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="F107" s="28" t="n">
+      <c r="F109" s="28" t="n">
         <v>3.27</v>
       </c>
-      <c r="G107" s="17" t="inlineStr">
+      <c r="G109" s="17" t="inlineStr">
         <is>
           <t>LNG선 4척 추가 수주를 통한 신규 수주 물량 확보.</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="15" customHeight="1" s="15">
-      <c r="A108" s="31" t="inlineStr">
+    <row r="110" ht="15" customHeight="1" s="15">
+      <c r="A110" s="31" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B108" s="31" t="inlineStr">
+      <c r="B110" s="31" t="inlineStr">
         <is>
           <t>영풍</t>
         </is>
       </c>
-      <c r="C108" s="31" t="inlineStr">
+      <c r="C110" s="31" t="inlineStr">
         <is>
           <t>KOSPI</t>
         </is>
       </c>
-      <c r="D108" s="35" t="inlineStr">
+      <c r="D110" s="35" t="inlineStr">
         <is>
           <t>금속</t>
         </is>
       </c>
-      <c r="E108" s="14" t="inlineStr">
+      <c r="E110" s="14" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="F108" s="28" t="n">
+      <c r="F110" s="28" t="n">
         <v>0.3</v>
       </c>
-      <c r="G108" s="17" t="inlineStr">
+      <c r="G110" s="17" t="inlineStr">
         <is>
           <t>계열사의 북미 빅테크향 고다층 인쇄회로기판 공급 계약.</t>
         </is>
       </c>
     </row>
-    <row r="109"/>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
+    <row r="111"/>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>다음 주 프리뷰</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr"/>
-      <c r="D110" s="3" t="inlineStr"/>
-      <c r="E110" s="3" t="inlineStr"/>
-      <c r="F110" s="3" t="inlineStr"/>
-      <c r="G110" s="3" t="inlineStr"/>
-      <c r="H110" s="3" t="inlineStr"/>
-      <c r="I110" s="3" t="inlineStr"/>
-      <c r="J110" s="3" t="inlineStr"/>
-      <c r="K110" s="3" t="inlineStr"/>
-    </row>
-    <row r="111" ht="15" customHeight="1" s="15">
-      <c r="A111" s="17" t="inlineStr">
-        <is>
-          <t>- 반도체 섹터 외국인 매도 진정 시 기술적 반등 전개</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="15" customHeight="1" s="15">
-      <c r="A112" s="17" t="inlineStr">
-        <is>
-          <t>- AI 속도조절론 지속에 따른 외국인 추가 이탈 시 하방 압력 확대</t>
-        </is>
-      </c>
+      <c r="C112" s="3" t="inlineStr"/>
+      <c r="D112" s="3" t="inlineStr"/>
+      <c r="E112" s="3" t="inlineStr"/>
+      <c r="F112" s="3" t="inlineStr"/>
+      <c r="G112" s="3" t="inlineStr"/>
+      <c r="H112" s="3" t="inlineStr"/>
+      <c r="I112" s="3" t="inlineStr"/>
+      <c r="J112" s="3" t="inlineStr"/>
+      <c r="K112" s="3" t="inlineStr"/>
     </row>
     <row r="113" ht="15" customHeight="1" s="15">
       <c r="A113" s="17" t="inlineStr">
         <is>
-          <t>- 외국인의 반도체 섹터 순매수 전환 여부</t>
+          <t>- 외국인 매도세 진정 및 반도체 대형주 수급 개선 시 지수 기술적 반등 전개</t>
         </is>
       </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="15">
       <c r="A114" s="17" t="inlineStr">
         <is>
-          <t>- FOMC 기준금리 결정</t>
+          <t>- AI 속도조절론 지속 및 외국인 매도세 지속 시 추가 하방 압력 발생</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="15">
       <c r="A115" s="17" t="inlineStr">
         <is>
-          <t>- 무역수지</t>
+          <t>- 외국인의 반도체 대형주 순매수 전환 여부</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="15">
       <c r="A116" s="17" t="inlineStr">
         <is>
-          <t>- 미국 소매판매</t>
+          <t>- 무역수지 및 수출입 확정치(9/15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="15" customHeight="1" s="15">
+      <c r="A117" s="17" t="inlineStr">
+        <is>
+          <t>- 미국 FOMC 기준금리 결정(9/17)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="52">
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A114:K114"/>
     <mergeCell ref="G105:K105"/>
@@ -3465,39 +3472,40 @@
     <mergeCell ref="A69:E69"/>
     <mergeCell ref="A65:E65"/>
     <mergeCell ref="A78:E78"/>
-    <mergeCell ref="G103:K103"/>
     <mergeCell ref="I1:K1"/>
-    <mergeCell ref="A99:K99"/>
     <mergeCell ref="A75:E75"/>
     <mergeCell ref="G69:K69"/>
     <mergeCell ref="A37:K37"/>
     <mergeCell ref="G87:K87"/>
     <mergeCell ref="A89:K89"/>
     <mergeCell ref="G83:K83"/>
+    <mergeCell ref="A101:K101"/>
     <mergeCell ref="G108:K108"/>
     <mergeCell ref="A95:K95"/>
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="G33:K33"/>
     <mergeCell ref="A113:K113"/>
-    <mergeCell ref="G104:K104"/>
     <mergeCell ref="G65:K65"/>
+    <mergeCell ref="G110:K110"/>
     <mergeCell ref="G79:K79"/>
     <mergeCell ref="A116:K116"/>
     <mergeCell ref="G73:K73"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A97:K97"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="A100:K100"/>
     <mergeCell ref="A96:K96"/>
+    <mergeCell ref="G109:K109"/>
     <mergeCell ref="G85:K85"/>
-    <mergeCell ref="A112:K112"/>
     <mergeCell ref="G32:K32"/>
     <mergeCell ref="A38:K38"/>
     <mergeCell ref="A115:K115"/>
+    <mergeCell ref="A117:K117"/>
     <mergeCell ref="A93:K93"/>
     <mergeCell ref="G106:K106"/>
     <mergeCell ref="C4:K4"/>
+    <mergeCell ref="A102:K102"/>
     <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A111:K111"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10196,7 +10204,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2032545E-31CB-476A-9A50-C610257E2F0C}</x14:id>
+          <x14:id>{CEC25292-303F-4ED8-B2DD-6FBE6AFD0998}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10210,7 +10218,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AAB57F4F-0CE1-4F07-B9CB-5D5E52CBCB20}</x14:id>
+          <x14:id>{53793DF9-B62B-405F-8151-B7EC148EA032}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10224,7 +10232,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3D87C0C5-28A2-45A3-86C0-B1FFEA6295E3}</x14:id>
+          <x14:id>{863BFD9F-EB08-4A7B-8250-41FAA248D6DB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10238,7 +10246,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{193057F8-B4A1-4044-82E1-6FE10A9D496F}</x14:id>
+          <x14:id>{B30D9CB4-9A45-4B18-B899-D6DD8F565016}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10248,7 +10256,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2032545E-31CB-476A-9A50-C610257E2F0C}">
+          <x14:cfRule type="dataBar" id="{CEC25292-303F-4ED8-B2DD-6FBE6AFD0998}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10261,7 +10269,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AAB57F4F-0CE1-4F07-B9CB-5D5E52CBCB20}">
+          <x14:cfRule type="dataBar" id="{53793DF9-B62B-405F-8151-B7EC148EA032}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10274,7 +10282,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3D87C0C5-28A2-45A3-86C0-B1FFEA6295E3}">
+          <x14:cfRule type="dataBar" id="{863BFD9F-EB08-4A7B-8250-41FAA248D6DB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10287,7 +10295,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{193057F8-B4A1-4044-82E1-6FE10A9D496F}">
+          <x14:cfRule type="dataBar" id="{B30D9CB4-9A45-4B18-B899-D6DD8F565016}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>